<commit_message>
Fill in missing English name for row 91
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JZTqyfR91E7Q7E4HBQmA45
</commit_message>
<xml_diff>
--- a/student_names_matched.xlsx
+++ b/student_names_matched.xlsx
@@ -565,7 +565,6 @@
           <t>KATAKORN</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -604,7 +603,6 @@
           <t>KHANTAPONG</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -643,7 +641,6 @@
           <t>KARANPAT</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -682,7 +679,6 @@
           <t>JITTAPAT</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -721,7 +717,6 @@
           <t>CHADAPORN</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -760,7 +755,6 @@
           <t>NAPHAT</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -804,7 +798,6 @@
           <t>NICHAKARN</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -843,7 +836,6 @@
           <t>THANON</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -882,7 +874,6 @@
           <t>NUNNAPAS</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -921,7 +912,6 @@
           <t>NATITHORN</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -960,7 +950,6 @@
           <t>BUSSAYARAT</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -999,7 +988,6 @@
           <t>PATIPOL</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -1038,7 +1026,6 @@
           <t>PUNNAKARN</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -1077,7 +1064,6 @@
           <t>PANSA</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -1116,7 +1102,6 @@
           <t>PHICHAYAPHA</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -1155,7 +1140,6 @@
           <t>PATTARAKIET</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -1194,7 +1178,6 @@
           <t>PAKIN</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -1233,7 +1216,6 @@
           <t>PADECH</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -1277,7 +1259,6 @@
           <t>PASINEE</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -1316,7 +1297,6 @@
           <t>MONRADA</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -1355,7 +1335,6 @@
           <t>WASAPHON</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -1394,7 +1373,6 @@
           <t>WISSUTA</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -1433,7 +1411,6 @@
           <t>SASIYAKORN</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -1472,7 +1449,6 @@
           <t>SIRADA</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -1511,7 +1487,6 @@
           <t>SIWANARD</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -1550,7 +1525,6 @@
           <t>SUPISARA</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="C27" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -1589,7 +1563,6 @@
           <t>SURAPAT</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="C28" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -1628,7 +1601,6 @@
           <t>ANGKACHAT</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="C29" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -1667,7 +1639,6 @@
           <t>THANYAPORN</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="C30" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -1706,7 +1677,6 @@
           <t>BENYAPA</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
       <c r="C31" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -1750,7 +1720,6 @@
           <t>VACHARAPOOM</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
       <c r="C32" s="1" t="inlineStr">
         <is>
           <t>Class5</t>
@@ -1789,7 +1758,6 @@
           <t>SURAWIN</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
       <c r="C33" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -1828,7 +1796,6 @@
           <t>KAMOLCHANOK</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
       <c r="C34" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -1867,7 +1834,6 @@
           <t>KRITSAKORN</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
       <c r="C35" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -1906,7 +1872,6 @@
           <t>GEDNAPA</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
       <c r="C36" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -1945,7 +1910,6 @@
           <t>JANEJIRA</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
       <c r="C37" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -1984,7 +1948,6 @@
           <t>THITIYA</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
       <c r="C38" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2023,7 +1986,6 @@
           <t>THIRAPORN</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr"/>
       <c r="C39" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2062,7 +2024,6 @@
           <t>NAPAT</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
       <c r="C40" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2106,7 +2067,6 @@
           <t>NUTCHA</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
       <c r="C41" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2145,7 +2105,6 @@
           <t>NATTHANON</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr"/>
       <c r="C42" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2184,7 +2143,6 @@
           <t>TANLUCK</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr"/>
       <c r="C43" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2223,7 +2181,6 @@
           <t>NUTCHANUN</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr"/>
       <c r="C44" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2267,7 +2224,6 @@
           <t>BANTITA</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr"/>
       <c r="C45" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2306,7 +2262,6 @@
           <t>BHANDER</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr"/>
       <c r="C46" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2345,7 +2300,6 @@
           <t>BENYAPA</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
       <c r="C47" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2389,7 +2343,6 @@
           <t>PANOTRAT</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr"/>
       <c r="C48" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2428,7 +2381,6 @@
           <t>PRAN</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr"/>
       <c r="C49" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2467,7 +2419,6 @@
           <t>PANISA</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
       <c r="C50" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2506,7 +2457,6 @@
           <t>PAIRAYA</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
       <c r="C51" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2545,7 +2495,6 @@
           <t>PHOPPOL</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr"/>
       <c r="C52" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2584,7 +2533,6 @@
           <t>PALATH</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr"/>
       <c r="C53" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2628,7 +2576,6 @@
           <t>PICHAYA</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr"/>
       <c r="C54" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2667,7 +2614,6 @@
           <t>PHUDIT</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr"/>
       <c r="C55" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2706,7 +2652,6 @@
           <t>PHUMPORN</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr"/>
       <c r="C56" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2745,7 +2690,6 @@
           <t>YOSSINEE</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr"/>
       <c r="C57" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2784,7 +2728,6 @@
           <t>WACHIRADA</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr"/>
       <c r="C58" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2823,7 +2766,6 @@
           <t>SUCHAYA</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr"/>
       <c r="C59" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2862,7 +2804,6 @@
           <t>SUWAPHAT</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr"/>
       <c r="C60" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2906,7 +2847,6 @@
           <t>SETTHAWUTH</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr"/>
       <c r="C61" s="1" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2945,7 +2885,6 @@
           <t>UTJIMA</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr"/>
       <c r="C62" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -2984,7 +2923,6 @@
           <t>HAMEEDA</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr"/>
       <c r="C63" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3023,7 +2961,6 @@
           <t>PANNAWAT</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr"/>
       <c r="C64" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3062,7 +2999,6 @@
           <t>SURAPOB</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr"/>
       <c r="C65" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3101,7 +3037,6 @@
           <t>KAMOLCHON</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr"/>
       <c r="C66" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3140,7 +3075,6 @@
           <t>KASEMSAN</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr"/>
       <c r="C67" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3179,7 +3113,6 @@
           <t>KHWANKAMOL</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
       <c r="C68" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3218,7 +3151,6 @@
           <t>JOAMKUAN</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr"/>
       <c r="C69" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3257,7 +3189,6 @@
           <t>CHANAKUL</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr"/>
       <c r="C70" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3296,7 +3227,6 @@
           <t>CHAVIS</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr"/>
       <c r="C71" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3335,7 +3265,6 @@
           <t>YANISA</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr"/>
       <c r="C72" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3374,7 +3303,6 @@
           <t>TANICHA</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr"/>
       <c r="C73" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3413,7 +3341,6 @@
           <t>THANIKA</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr"/>
       <c r="C74" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3452,7 +3379,6 @@
           <t>NATTHANICHA</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr"/>
       <c r="C75" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3491,7 +3417,6 @@
           <t>THANACHOT</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr"/>
       <c r="C76" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3530,7 +3455,6 @@
           <t>THANAPHON</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr"/>
       <c r="C77" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3569,7 +3493,6 @@
           <t>THANANYA</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr"/>
       <c r="C78" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3608,7 +3531,6 @@
           <t>NANCHAYA</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr"/>
       <c r="C79" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3647,7 +3569,6 @@
           <t>NICHANANT</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr"/>
       <c r="C80" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3686,7 +3607,6 @@
           <t>PUNYAVEE</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr"/>
       <c r="C81" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3725,7 +3645,6 @@
           <t>PHOLLAWAT</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr"/>
       <c r="C82" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3769,7 +3688,6 @@
           <t>PIMCHANOKE</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr"/>
       <c r="C83" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3808,7 +3726,6 @@
           <t>PAKAPORN</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr"/>
       <c r="C84" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3847,7 +3764,6 @@
           <t>PAKPRAPA</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr"/>
       <c r="C85" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3886,7 +3802,6 @@
           <t>PATTHARAKORN</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr"/>
       <c r="C86" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3925,7 +3840,6 @@
           <t>RAPEEPAT</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr"/>
       <c r="C87" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -3964,7 +3878,6 @@
           <t>SUPARADA</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr"/>
       <c r="C88" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -4003,7 +3916,6 @@
           <t>SUVAPICH</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr"/>
       <c r="C89" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -4042,7 +3954,6 @@
           <t>ATHIKAN</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr"/>
       <c r="C90" s="2" t="inlineStr">
         <is>
           <t>Class4</t>
@@ -4076,9 +3987,16 @@
       </c>
     </row>
     <row r="91" ht="20.4" customHeight="1" thickBot="1">
-      <c r="A91" s="10" t="n"/>
-      <c r="B91" t="inlineStr"/>
-      <c r="C91" s="2" t="n"/>
+      <c r="A91" s="9" t="inlineStr">
+        <is>
+          <t>ORNANONG</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Class4</t>
+        </is>
+      </c>
       <c r="F91" s="8" t="n">
         <v>66200070</v>
       </c>
@@ -4107,7 +4025,7 @@
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>ไม่พบชื่อภาษาอังกฤษของคนนี้ในรายการเดิม</t>
+          <t>ชื่ออังกฤษเดาจากการออกเสียง (ไม่มีในรายการเดิม) ควรตรวจสอบกับเจ้าของชื่อ</t>
         </is>
       </c>
     </row>
@@ -4117,7 +4035,6 @@
           <t>ATTAKITT</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr"/>
       <c r="C92" s="2" t="inlineStr">
         <is>
           <t>Class4</t>

</xml_diff>